<commit_message>
Corregir la zona horaria a Colombia
La documentación decía America/Mexico_City por un supuesto mío, pero la
familia está en Bogotá. Una zona horaria equivocada haría que los
recordatorios se disparen con una hora de diferencia, que es el tipo de
fallo que nadie nota hasta que alguien toma una pastilla a destiempo.

Actualiza SETUP.md, la hoja Config y la pestaña Leeme del Excel, y cambia
el formato de fechas de la interfaz de es-MX a es-CO.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PillTime-DB.xlsx
+++ b/PillTime-DB.xlsx
@@ -565,7 +565,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>En Apps Script ve a Configuración del proyecto y pon la zona horaria correcta (America/Mexico_City).</t>
+          <t>En Apps Script ve a Configuración del proyecto y pon la zona horaria correcta (America/Bogota).</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>America/Mexico_City</t>
+          <t>America/Bogota</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">

</xml_diff>